<commit_message>
Envoy 3.1: warm stone look, round shields, Pilzholz instead of Quarz
- Palette moved from iron and steel to stone, earth and copper: warm
  stone panels with copper corner fittings, copper buttons, a carved
  stone ledge with a copper inlay for the menu
- Menu buttons are round shields: copper rim with rivets, a face of
  stone, the emblem carved into it; locked ones carry a copper lock
- Pilzholz replaces Quarz as the light material that is worked like
  wood: stems of the giant fungi at the new Pilzhain; quartz from older
  expeditions still counts as Pilzholz
- Map re-drawn in sepia with giant mushrooms, homes in warm stone with
  lit windows, round app icon with a carved E, warmer base figure
- Spec, CLAUDE.md and the xlsx explanations updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117M4aYJ5RoPwj7oU8m6XcB
</commit_message>
<xml_diff>
--- a/data/welt.xlsx
+++ b/data/welt.xlsx
@@ -550,12 +550,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>quarzhang</t>
+          <t>pilzhain</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Quarzhang</t>
+          <t>Pilzhain</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -583,7 +583,7 @@
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Helle Kristalle wachsen aus dem Geröll, kalt und klar.</t>
+          <t>Zwischen den Trümmern stehen Pilze, hoch wie Säulen. Ihre Stiele sind leicht und zäh.</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>aether:3-5, quarz:0-1, item:5</t>
+          <t>aether:3-5, pilzholz:0-1, item:5</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>aether:5-9, quarz:0-2, item:8</t>
+          <t>aether:5-9, pilzholz:0-2, item:8</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -1883,17 +1883,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>q-quarz</t>
+          <t>q-pilzholz</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Quarz brechen</t>
+          <t>Pilzholz schlagen</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>quarzhang</t>
+          <t>pilzhain</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Klare Kristalle aus dem Geröll lösen.</t>
+          <t>Einen Stiel fällen und in leichte, handliche Stücke teilen.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
@@ -1927,7 +1927,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>quarz:2-4</t>
+          <t>pilzholz:2-4</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -2039,7 +2039,7 @@
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>quarz:6, stein:6</t>
+          <t>pilzholz:6, stein:6</t>
         </is>
       </c>
       <c r="L4" s="2" t="n">
@@ -2459,7 +2459,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Mit Stein, Quarz und einem langen Atem lässt sich die Brücke neu legen.</t>
+          <t>Mit Pilzholz, Stein und einem langen Atem lässt sich die Brücke neu legen.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr"/>
@@ -2479,7 +2479,7 @@
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>quarz:10, stein:12</t>
+          <t>pilzholz:10, stein:12</t>
         </is>
       </c>
       <c r="L11" s="2" t="n">
@@ -2855,7 +2855,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>quarz</t>
+          <t>pilzholz</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Feste Mauern, Fenster aus Quarz, die das Licht weich machen.</t>
+          <t>Feste Mauern, Balken aus Pilzholz, ein Dach, das hält.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -3626,7 +3626,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>lager (Ausgangspunkt jeder Expedition, dort steht das Zuhause), wild (Geister tauchen auf), sammeln (Quarz oder Stein), hoehle (mehrere Geister nacheinander), ort (feste Quests).</t>
+          <t>lager (Ausgangspunkt jeder Expedition, dort steht das Zuhause), wild (Geister tauchen auf), sammeln (Pilzholz oder Stein), hoehle (mehrere Geister nacheinander), ort (feste Quests).</t>
         </is>
       </c>
     </row>
@@ -3718,7 +3718,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>aether:2-4, quarz:0-1, stein:0-1, item:5 (Prozent-Chance auf ein Ausrüstungsteil).</t>
+          <t>aether:2-4, pilzholz:0-1, stein:0-1, item:5 (Prozent-Chance auf ein Ausrüstungsteil).</t>
         </is>
       </c>
     </row>
@@ -3798,7 +3798,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Material, das die Quest verbraucht: quarz:6, stein:6.</t>
+          <t>Material, das die Quest verbraucht: pilzholz:6, stein:6.</t>
         </is>
       </c>
     </row>
@@ -3822,7 +3822,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>aether:20, quarz:2-4, stein:1-3, item:&lt;id&gt;, einrichtung:&lt;id&gt;, freischaltung:zuhause oder haendler, rast:1 (Leiste voll). Bei Höhlen nur, wenn alle Geister bezwungen sind.</t>
+          <t>aether:20, pilzholz:2-4, stein:1-3, item:&lt;id&gt;, einrichtung:&lt;id&gt;, freischaltung:zuhause oder haendler, rast:1 (Leiste voll). Bei Höhlen nur, wenn alle Geister bezwungen sind.</t>
         </is>
       </c>
     </row>
@@ -3849,7 +3849,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>quarz, stein, aether</t>
+          <t>pilzholz, stein, aether</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Envoy 3.3: palette after the reference image, veins, Bannsplitter
- Palette taken from the reference: dark petrol stone, ivory, burnt
  orange and a dusty blue; no brown, no sepia
- Organic veins: a seamless vein texture over the panels and fine veins
  on the faces of the round shields; the chosen shield turns ivory
- Currency renamed from Traumsplitter to Bannsplitter (what remains when
  a spirit is banished); texts now read the name from CURRENCY
- Map in ivory and dusty blue with orange mushrooms and an ember glow
  at the Aschenhang; homes in blue-grey stone with orange windows; app
  icon as an ivory disc with veins and an orange rim
- Spec and CLAUDE.md updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117M4aYJ5RoPwj7oU8m6XcB
</commit_message>
<xml_diff>
--- a/data/welt.xlsx
+++ b/data/welt.xlsx
@@ -3559,7 +3559,7 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Eine Schale voller Traumsplitter, die nie ganz erlöschen.</t>
+          <t>Eine Schale voller Bannsplitter, die nie ganz erlöschen.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -3706,7 +3706,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>ja = mit Gelassenheit kann der Geist beruhigt statt besiegt werden (mehr Traumsplitter).</t>
+          <t>ja = mit Gelassenheit kann der Geist beruhigt statt besiegt werden (mehr Bannsplitter).</t>
         </is>
       </c>
     </row>
@@ -3786,7 +3786,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Werte, die mehr Ertrag bringen (beim Sammeln +1 je 3 Level, sonst +5 % Traumsplitter je Level).</t>
+          <t>Werte, die mehr Ertrag bringen (beim Sammeln +1 je 3 Level, sonst +5 % Bannsplitter je Level).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Envoy 3.5: time follows stamina, many quick quests, a few long ones
Every point of stamina is one minute away from the camp: ways and the
work on site cost stamina and take as many minutes. Near places are one
minute away, so the quickest quests take three minutes; long ones take
an hour or more and need a long bar. The bar is 20 + 4 per Ausdauer.

New quests: small, medium and large gathering at the Pilzhain and the
Steinbruch, Bannsplitter from the shore gravel, and three long
repeatable quests. Yields are smaller and home tiers cost more, so the
quick quests do not open everything in a few days. A build keeps the
price it had, so an existing home stays. Gathering bonus is now +5 %
per level, rounded by chance, and the last minute of a trip counts
down in seconds.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117M4aYJ5RoPwj7oU8m6XcB
</commit_message>
<xml_diff>
--- a/data/welt.xlsx
+++ b/data/welt.xlsx
@@ -1777,25 +1777,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="7" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
-    <col width="50" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1836,45 +1835,40 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>dauer</t>
+          <t>tempo</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>tempo</t>
+          <t>ertrag</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>ertrag</t>
+          <t>verbrauch</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>verbrauch</t>
+          <t>kosten</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>kosten</t>
+          <t>belohnung</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>belohnung</t>
+          <t>wiederholbar</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>wiederholbar</t>
+          <t>abklingzeit</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>abklingzeit</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>notiz</t>
         </is>
@@ -1883,12 +1877,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>q-pilzholz</t>
+          <t>q-pilzholz-klein</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Pilzholz schlagen</t>
+          <t>Pilzholz auflesen</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1903,57 +1897,50 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Einen Stiel fällen und in leichte, handliche Stücke teilen.</t>
+          <t>Was der Wind von den Hüten gebrochen hat, liegt leicht im Moos.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="n">
-        <v>15</v>
-      </c>
+      <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>kraft, ausdauer</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
           <t>kraft</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="n">
-        <v>2</v>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>pilzholz:1</t>
+        </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>pilzholz:2-4</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
           <t>ja</t>
         </is>
       </c>
-      <c r="O2" s="2" t="n">
+      <c r="N2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="P2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>q-stein</t>
+          <t>q-pilzholz</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Steine brechen</t>
+          <t>Pilzholz schlagen</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>steinbruch</t>
+          <t>pilzhain</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1963,73 +1950,76 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Lose Blöcke lösen und handlich schlagen.</t>
+          <t>Einen Stiel fällen und in leichte, handliche Stücke teilen.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
       <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="n">
-        <v>15</v>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>kraft, ausdauer</t>
+        </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
           <t>kraft</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>kraft</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="n">
-        <v>2</v>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>pilzholz:2-3</t>
+        </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>stein:2-4</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
           <t>ja</t>
         </is>
       </c>
-      <c r="O3" s="2" t="n">
+      <c r="N3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="P3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>q-zuhause</t>
+          <t>q-pilzholz-gross</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Ein Platz zum Bleiben</t>
+          <t>Einen Riesenpilz fällen</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>lager</t>
+          <t>pilzhain</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>bauen</t>
+          <t>sammeln</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Zwischen den Säulen ist Platz für ein Zelt. Es fehlt nur das Material.</t>
+          <t>Ein ganzer Stamm, so hoch wie eine Säule. Das Holz reicht für eine Wand.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="n">
-        <v>30</v>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>kraft&gt;=4</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>kraft, ausdauer</t>
+        </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -2037,291 +2027,266 @@
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>pilzholz:6, stein:6</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="n">
-        <v>2</v>
+      <c r="K4" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>pilzholz:7-9</t>
+        </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>freischaltung:zuhause, splitter:10</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>nein</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="n">
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="P4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>q-saeule</t>
+          <t>q-stein-klein</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Die umgestürzte Säule</t>
+          <t>Lose Steine auflesen</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>stillesufer</t>
+          <t>steinbruch</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>erkunden</t>
+          <t>sammeln</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Eine Säule liegt quer über dem Pfad. Wer sie zerlegt, hat Stein für Tage.</t>
+          <t>Am Rand des Bruchs liegt, was von allein herabgefallen ist.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>kraft&gt;=3</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>20</v>
-      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr">
         <is>
           <t>kraft</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>kraft</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="n">
-        <v>2</v>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>stein:1</t>
+        </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>stein:4-6, splitter:4</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
           <t>ja</t>
         </is>
       </c>
-      <c r="O5" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="P5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>q-haendler</t>
+          <t>q-stein</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Der Händler im Nebel</t>
+          <t>Steine brechen</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>nebelfurt</t>
+          <t>steinbruch</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>kampf</t>
+          <t>sammeln</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>In der Furt ruft jemand um Hilfe. Ein Wagen steckt fest, und davor steht etwas Großes.</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>nebelwaechter</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>kraft&gt;=3, ausdauer&gt;=3</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="I6" s="2" t="inlineStr"/>
+          <t>Lose Blöcke lösen und handlich schlagen.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>kraft</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>kraft</t>
+        </is>
+      </c>
       <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="n">
-        <v>3</v>
+      <c r="K6" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>stein:2-3</t>
+        </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>freischaltung:haendler, splitter:25</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>nein</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="n">
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="P6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>q-echohoehle</t>
+          <t>q-stein-gross</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Die Echohöhle</t>
+          <t>Einen Block lösen</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>echohoehle</t>
+          <t>steinbruch</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>hoehle</t>
+          <t>sammeln</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Tief drinnen hausen fünf Geister. Wie weit der Envoy kommt, hängt an seinen Werten.</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>zauderling, nebelwicht, gruebelkraehe, hastwind, dornenfluesterer</t>
-        </is>
-      </c>
+          <t>Ein Block aus der Wand, sauber gespalten. Schwer, aber er trägt ein Haus.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>kraft&gt;=2</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I7" s="2" t="inlineStr"/>
+          <t>kraft&gt;=5</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>kraft</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>kraft</t>
+        </is>
+      </c>
       <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="n">
-        <v>3</v>
+      <c r="K7" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>stein:7-9</t>
+        </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>splitter:30, item:beine_kampfhose_2</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
           <t>ja</t>
         </is>
       </c>
-      <c r="O7" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="P7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>q-spalt</t>
+          <t>q-zuhause</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Durch den Spalt</t>
+          <t>Ein Platz zum Bleiben</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>spalt</t>
+          <t>lager</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>erkunden</t>
+          <t>bauen</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Dahinter soll ein Versteck liegen. Hindurch passt nur, wer sich drehen und strecken kann.</t>
+          <t>Zwischen den Säulen ist Platz für ein Zelt. Es fehlt nur das Material.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>beweglichkeit&gt;=4</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>beweglichkeit</t>
-        </is>
-      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>kraft</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>beweglichkeit</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="n">
-        <v>2</v>
+          <t>pilzholz:6, stein:6</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>freischaltung:zuhause, splitter:10</t>
+        </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>splitter:15, item:kopf_stirnband_1</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
           <t>nein</t>
         </is>
       </c>
-      <c r="O8" s="2" t="n">
+      <c r="N8" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="P8" s="2" t="inlineStr"/>
+      <c r="O8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>q-quelle</t>
+          <t>q-uferkies</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Die stille Quelle</t>
+          <t>Splitter im Uferkies</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>stillequelle</t>
+          <t>stillesufer</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -2331,61 +2296,50 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Wer am Rand sitzen bleibt, bis das Wasser ganz ruhig ist, steht erholt wieder auf.</t>
+          <t>Wo früher Geister gebannt wurden, glimmen noch Splitter zwischen den Kieseln.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>gelassenheit&gt;=3</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>25</v>
-      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr">
         <is>
           <t>gelassenheit</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>gelassenheit</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="n">
-        <v>1</v>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>splitter:1</t>
+        </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>splitter:8, rast:1</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
           <t>ja</t>
         </is>
       </c>
-      <c r="O9" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="P9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>q-dornen</t>
+          <t>q-saeule</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Über den Dornengrat</t>
+          <t>Die umgestürzte Säule</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>dornengrat</t>
+          <t>stillesufer</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -2395,249 +2349,233 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Der Grat flüstert. Hinüber kommt, wer sich weder hetzen noch festhalten lässt.</t>
+          <t>Eine Säule liegt quer über dem Pfad. Wer sie zerlegt, hat Stein für Tage.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr"/>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>beweglichkeit&gt;=5, gelassenheit&gt;=4</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>30</v>
+          <t>kraft&gt;=3</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>kraft</t>
+        </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>beweglichkeit</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>gelassenheit</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="n">
+          <t>kraft</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>stein:4-6, splitter:4</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>splitter:20, einrichtung:windspiel</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>nein</t>
-        </is>
-      </c>
-      <c r="O10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>q-bruecke</t>
+          <t>q-haendler</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Die Brücke über die Schlucht</t>
+          <t>Der Händler im Nebel</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>schlucht</t>
+          <t>nebelfurt</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>bauen</t>
+          <t>kampf</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Mit Pilzholz, Stein und einem langen Atem lässt sich die Brücke neu legen.</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr"/>
+          <t>In der Furt ruft jemand um Hilfe. Ein Wagen steckt fest, und davor steht etwas Großes.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>nebelwaechter</t>
+        </is>
+      </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>ausdauer&gt;=5, kraft&gt;=4</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>kraft, ausdauer</t>
-        </is>
-      </c>
+          <t>kraft&gt;=3, ausdauer&gt;=3</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>pilzholz:10, stein:12</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="n">
-        <v>4</v>
+      <c r="K11" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>freischaltung:haendler, splitter:25</t>
+        </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>splitter:30</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
           <t>nein</t>
         </is>
       </c>
-      <c r="O11" s="2" t="n">
+      <c r="N11" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="P11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>q-mondsee</t>
+          <t>q-furtwache</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Spiegel im Mondsee</t>
+          <t>Wache an der Furt</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>mondsee</t>
+          <t>nebelfurt</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>kampf</t>
+          <t>erkunden</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Im Wasser steht jemand, der nur wiederholt, was man selbst einmal gesagt hat.</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>echo</t>
-        </is>
-      </c>
+          <t>Lange am Wasser sitzen, bis der Nebel zeigt, was er mit sich trägt.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>gelassenheit&gt;=6</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="I12" s="2" t="inlineStr"/>
+          <t>gelassenheit&gt;=5</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>gelassenheit</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>gelassenheit</t>
+        </is>
+      </c>
       <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="n">
-        <v>3</v>
+      <c r="K12" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>splitter:9-12</t>
+        </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>splitter:35, item:kopf_stillemaske_3</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>nein</t>
-        </is>
-      </c>
-      <c r="O12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" s="2" t="inlineStr"/>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>q-turm</t>
+          <t>q-echohoehle</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Der Turm der Stufen</t>
+          <t>Die Echohöhle</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>turm</t>
+          <t>echohoehle</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>erkunden</t>
+          <t>hoehle</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Oben soll man weit sehen. Wer im echten Leben genug Stufen gegangen ist, kennt den Rhythmus.</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr"/>
+          <t>Tief drinnen hausen fünf Geister. Wie weit der Envoy kommt, hängt an seinen Werten.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>zauderling, nebelwicht, gruebelkraehe, hastwind, dornenfluesterer</t>
+        </is>
+      </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>summe_stockwerke&gt;=100</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>ausdauer</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>ausdauer</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="n">
-        <v>4</v>
+          <t>kraft&gt;=2</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>splitter:30, item:beine_kampfhose_2</t>
+        </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>splitter:60, item:schuhe_leichtestiefel_3</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>nein</t>
-        </is>
-      </c>
-      <c r="O13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="2" t="inlineStr"/>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>q-langestrasse</t>
+          <t>q-spalt</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Die lange Straße</t>
+          <t>Durch den Spalt</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>langestrasse</t>
+          <t>spalt</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -2647,173 +2585,648 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Die Straße endet nur für die, die schon viele Kilometer in den Beinen haben.</t>
+          <t>Dahinter soll ein Versteck liegen. Hindurch passt nur, wer sich drehen und strecken kann.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>summe_km&gt;=30</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>40</v>
+          <t>beweglichkeit&gt;=4</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>beweglichkeit</t>
+        </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>ausdauer</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>ausdauer</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="n">
-        <v>4</v>
+          <t>beweglichkeit</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>splitter:15, item:kopf_stirnband_1</t>
+        </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>splitter:40</t>
-        </is>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
           <t>nein</t>
         </is>
       </c>
-      <c r="O14" s="2" t="n">
+      <c r="N14" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="P14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>q-aschenthron</t>
+          <t>q-quelle</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Der Aschenthron</t>
+          <t>Die stille Quelle</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>aschenhang</t>
+          <t>stillequelle</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>hoehle</t>
+          <t>erkunden</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Der Weg zum Thron führt an drei Wächtern vorbei. Oben sitzt sie, auf kalter Glut.</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>schwerer-schatten, glutfresser, glutfresser, aschenkoenigin</t>
-        </is>
-      </c>
+          <t>Wer am Rand sitzen bleibt, bis das Wasser ganz ruhig ist, steht erholt wieder auf.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr"/>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>kraft&gt;=8</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I15" s="2" t="inlineStr"/>
+          <t>gelassenheit&gt;=3</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>gelassenheit</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>gelassenheit</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="n">
-        <v>5</v>
+      <c r="K15" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>splitter:8, rast:1</t>
+        </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>splitter:120, item:handschuhe_nebelwickel_4, einrichtung:splitterschale</t>
-        </is>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>nein</t>
-        </is>
-      </c>
-      <c r="O15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" s="2" t="inlineStr"/>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>q-dornen</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Über den Dornengrat</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>dornengrat</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>erkunden</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Der Grat flüstert. Hinüber kommt, wer sich weder hetzen noch festhalten lässt.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>beweglichkeit&gt;=5, gelassenheit&gt;=4</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>beweglichkeit</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>gelassenheit</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>splitter:20, einrichtung:windspiel</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>q-bruecke</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Die Brücke über die Schlucht</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>schlucht</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>bauen</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Mit Pilzholz, Stein und einem langen Atem lässt sich die Brücke neu legen.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>ausdauer&gt;=5, kraft&gt;=4</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>kraft, ausdauer</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>pilzholz:10, stein:12</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>splitter:30</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>q-mondsee</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Spiegel im Mondsee</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>mondsee</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>kampf</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Im Wasser steht jemand, der nur wiederholt, was man selbst einmal gesagt hat.</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>echo</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>gelassenheit&gt;=6</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>splitter:35, item:kopf_stillemaske_3</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>q-mondnacht</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Eine Nacht am Mondsee</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>mondsee</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>erkunden</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Bis der Mond über das Wasser gewandert ist. Was dann im Uferschlamm liegt, hat lange gewartet.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>quest:q-mondsee</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>gelassenheit</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>gelassenheit</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>splitter:15-19</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>q-turm</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Der Turm der Stufen</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>turm</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>erkunden</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Oben soll man weit sehen. Wer im echten Leben genug Stufen gegangen ist, kennt den Rhythmus.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>summe_stockwerke&gt;=100</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>ausdauer</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>ausdauer</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>splitter:60, item:schuhe_leichtestiefel_3</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>q-langestrasse</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Die lange Straße</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>langestrasse</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>erkunden</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Die Straße endet nur für die, die schon viele Kilometer in den Beinen haben.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>summe_km&gt;=30</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>ausdauer</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>ausdauer</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>splitter:40</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>q-horizont</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Bis zum Horizont</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>langestrasse</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>erkunden</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Hinter dem Ende der Straße geht es weiter. Wer bis zum Abend läuft, kommt mit vollen Taschen zurück.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>quest:q-langestrasse</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>ausdauer</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>ausdauer</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>splitter:24-30</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>q-aschenthron</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Der Aschenthron</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>aschenhang</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>hoehle</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Der Weg zum Thron führt an drei Wächtern vorbei. Oben sitzt sie, auf kalter Glut.</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>schwerer-schatten, glutfresser, glutfresser, aschenkoenigin</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>kraft&gt;=8</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>splitter:120, item:handschuhe_nebelwickel_4, einrichtung:splitterschale</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t>q-leere</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Das weiße Schweigen</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>weisstal</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>kampf</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>Im Tal wartet etwas, das man nicht besiegen muss.</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>die-leere</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>gelassenheit&gt;=10</t>
         </is>
       </c>
-      <c r="H16" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
         <is>
           <t>splitter:200</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>nein</t>
         </is>
       </c>
-      <c r="O16" s="2" t="n">
+      <c r="N24" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="P16" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="D2:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"sammeln,erkunden,kampf,hoehle,bauen"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"ja,nein"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2942,13 +3355,13 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>10</v>
@@ -2980,13 +3393,13 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>15</v>
@@ -3018,13 +3431,13 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>50</v>
+        <v>180</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>250</v>
+        <v>450</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>22</v>
@@ -3056,13 +3469,13 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>50</v>
+        <v>180</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>80</v>
+        <v>300</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>500</v>
+        <v>900</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>30</v>
@@ -3579,7 +3992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3614,7 +4027,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Position auf der Karte in Prozent von Breite und Höhe (0 bis 100). Die Entfernung zum Lager bestimmt Reisezeit und Ausdauer.</t>
+          <t>Position auf der Karte in Prozent von Breite und Höhe (0 bis 100). Die Entfernung zum Lager bestimmt die Ausdauer für den Weg: 20 Einheiten Entfernung = 1 Ausdauer = 1 Minute.</t>
         </is>
       </c>
     </row>
@@ -3694,7 +4107,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Lebenspunkte, Schaden je Treffer, Geschick (gegen Beweglichkeit gewürfelt). Bestimmen, wie lange ein Kampf dauert.</t>
+          <t>Lebenspunkte, Schaden je Treffer, Geschick (gegen Beweglichkeit gewürfelt). Bestimmen, wie ein Kampf ausgeht.</t>
         </is>
       </c>
     </row>
@@ -3757,12 +4170,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>dauer</t>
+          <t>kosten</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Minuten vor Ort bei Werten auf 1. Bei Kampf und Höhle kommt die Kampfzeit dazu.</t>
+          <t>Ausdauer für die Arbeit vor Ort bei Werten auf 1. Jeder Punkt Ausdauer ist eine Minute: kosten 7 heißt 7 Minuten vor Ort. Hin- und Rückweg kommen nach Entfernung dazu.</t>
         </is>
       </c>
     </row>
@@ -3774,7 +4187,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Werte, die die Zeit vor Ort verkürzen (4 % je Level, höchstens auf die Hälfte).</t>
+          <t>Werte, die die Arbeit vor Ort kürzer und damit billiger machen (4 % je Level, höchstens auf die Hälfte).</t>
         </is>
       </c>
     </row>
@@ -3786,7 +4199,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Werte, die mehr Ertrag bringen (beim Sammeln +1 je 3 Level, sonst +5 % Bannsplitter je Level).</t>
+          <t>Werte, die mehr Ertrag bringen: +5 % je Level, beim Sammeln auf die Stücke, beim Erkunden auf die Bannsplitter.</t>
         </is>
       </c>
     </row>
@@ -3805,110 +4218,98 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>kosten</t>
+          <t>belohnung</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Ausdauer für die Arbeit vor Ort. Hin- und Rückweg kommen nach Entfernung dazu.</t>
+          <t>splitter:20, pilzholz:2-4, stein:1-3, item:&lt;id&gt;, einrichtung:&lt;id&gt;, freischaltung:zuhause oder haendler, rast:1 (Leiste voll). Bei Höhlen nur, wenn alle Geister bezwungen sind.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>belohnung</t>
+          <t>wiederholbar, abklingzeit</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>splitter:20, pilzholz:2-4, stein:1-3, item:&lt;id&gt;, einrichtung:&lt;id&gt;, freischaltung:zuhause oder haendler, rast:1 (Leiste voll). Bei Höhlen nur, wenn alle Geister bezwungen sind.</t>
+          <t>ja = kann erneut gemacht werden, frühestens nach so vielen Tagen.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>wiederholbar, abklingzeit</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>ja = kann erneut gemacht werden, frühestens nach so vielen Tagen.</t>
-        </is>
-      </c>
+          <t>ZUHAUSE</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ZUHAUSE</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr"/>
+          <t>pilzholz, stein, splitter</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Kosten für den Ausbau auf diese Stufe. Stufe 1 entsteht durch die Quest.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>pilzholz, stein, splitter</t>
+          <t>erholung</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Kosten für den Ausbau auf diese Stufe. Stufe 1 entsteht durch die Quest.</t>
+          <t>Prozent schneller füllt sich die Ausdauerleiste.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>erholung</t>
+          <t>plaetze, schrank</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Prozent schneller füllt sich die Ausdauerleiste.</t>
+          <t>Plätze für Einrichtung, Fächer im Schrank.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>plaetze, schrank</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>Plätze für Einrichtung, Fächer im Schrank.</t>
-        </is>
-      </c>
+          <t>EINRICHTUNG</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>EINRICHTUNG</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr"/>
+          <t>effekt</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>erholung:+5 und/oder glueck:+3 (Prozent).</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>effekt</t>
+          <t>ab_stufe</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>erholung:+5 und/oder glueck:+3 (Prozent).</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>ab_stufe</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Ab welcher Stufe des Zuhauses sie aufgestellt werden kann.</t>
         </is>

</xml_diff>

<commit_message>
Envoy 4.4: short bonus, bigger portrait, dark Tageswerk button, glowing menu
The bonus of the first achievement now lasts only the first 15 minutes
after the start, to get going right away. The Tageswerk page names it
with its end while it runs.

The quest that unlocks the camp extension is taken out for now (new
column aktiv in the quests table); the camp has no upgrade button until
the housing exists.

The top bar is on every page, also on the Envoy's own page (there
without the portrait) and in the Handbuch. The portrait is much bigger
and hangs into the page. The Tageswerk button is dark stone like the
menu, with a large orange glow that pulses while tasks are open.

A menu point with something new glows at its rim instead of showing a
dot, and stops when the section is opened. The lock on closed menu
points is a round, light silver seal.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117M4aYJ5RoPwj7oU8m6XcB
</commit_message>
<xml_diff>
--- a/data/welt.xlsx
+++ b/data/welt.xlsx
@@ -1777,7 +1777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1794,7 +1794,8 @@
     <col width="50" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1870,6 +1871,11 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
           <t>notiz</t>
         </is>
       </c>
@@ -1925,7 +1931,12 @@
       <c r="N2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1982,7 +1993,12 @@
       <c r="N3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2043,7 +2059,12 @@
       <c r="N4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2096,7 +2117,12 @@
       <c r="N5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O5" s="2" t="inlineStr"/>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2153,7 +2179,12 @@
       <c r="N6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2214,7 +2245,12 @@
       <c r="N7" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O7" s="2" t="inlineStr"/>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2271,7 +2307,12 @@
       <c r="N8" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O8" s="2" t="inlineStr"/>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2324,7 +2365,12 @@
       <c r="N9" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O9" s="2" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2385,7 +2431,12 @@
       <c r="N10" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="O10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2442,7 +2493,12 @@
       <c r="N11" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2503,7 +2559,12 @@
       <c r="N12" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="O12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2560,7 +2621,12 @@
       <c r="N13" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2621,7 +2687,12 @@
       <c r="N14" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2682,7 +2753,12 @@
       <c r="N15" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="O15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2743,7 +2819,12 @@
       <c r="N16" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O16" s="2" t="inlineStr"/>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2804,7 +2885,12 @@
       <c r="N17" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O17" s="2" t="inlineStr"/>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2861,7 +2947,12 @@
       <c r="N18" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2922,7 +3013,12 @@
       <c r="N19" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O19" s="2" t="inlineStr"/>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2983,7 +3079,12 @@
       <c r="N20" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3044,7 +3145,12 @@
       <c r="N21" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3105,7 +3211,12 @@
       <c r="N22" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="O22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3162,7 +3273,12 @@
       <c r="N23" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3219,14 +3335,22 @@
       <c r="N24" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="D2:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"sammeln,erkunden,kampf,hoehle,bauen"</formula1>
     </dataValidation>
     <dataValidation sqref="M2:M200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ja,nein"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"ja,nein"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3992,7 +4116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4242,74 +4366,86 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ZUHAUSE</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr"/>
+          <t>aktiv</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>nein = die Quest bleibt in der Tabelle, wird im Spiel aber vorerst nicht angeboten. Leer = ja.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>pilzholz, stein, splitter</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Kosten für den Ausbau auf diese Stufe. Stufe 1 entsteht durch die Quest.</t>
-        </is>
-      </c>
+          <t>ZUHAUSE</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>erholung</t>
+          <t>pilzholz, stein, splitter</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Prozent schneller füllt sich die Ausdauerleiste.</t>
+          <t>Kosten für den Ausbau auf diese Stufe. Stufe 1 entsteht durch die Quest.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>plaetze, schrank</t>
+          <t>erholung</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Plätze für Einrichtung, Fächer im Schrank.</t>
+          <t>Prozent schneller füllt sich die Ausdauerleiste.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>EINRICHTUNG</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr"/>
+          <t>plaetze, schrank</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Plätze für Einrichtung, Fächer im Schrank.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>effekt</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>erholung:+5 und/oder glueck:+3 (Prozent).</t>
-        </is>
-      </c>
+          <t>EINRICHTUNG</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>effekt</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>erholung:+5 und/oder glueck:+3 (Prozent).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>ab_stufe</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Ab welcher Stufe des Zuhauses sie aufgestellt werden kann.</t>
         </is>

</xml_diff>

<commit_message>
Test-Knöpfe nur in der Testfassung, Hygge als Zahl, Werte 1/1/2/3, Krempelplatz
- Testfassung: Kasten „Nur im Test“ im Vorrat (Lager, Abenteuer) mit
  „Energie auffüllen“, „+10 Stein“, „+10 Pilzholz“ (Ereignis test, Material
  nur so viel, wie passt); die echte Fassung zeigt ihn nie (stage.js)
- Hygge: nur die Zahl in einer runden Medaille, ohne Ring, Ziel und
  Einrichtungs-Zeichen; „Lager aufwerten“ glimmt, sobald das Hygge reicht
- Hygge-Werte: Steinlager 1, Pilzlager 1, Krempelplatz 2, Schlafplatz 3;
  Lagerstufe 2 ab 5 (welt.xlsx neu erzeugt, vorher unverändert geprüft)
- Aufbewahrung heißt auf Stufe 1 „Krempelplatz“ (Name je Stufe aus der Tabelle)
- Formen: Knöpfe auf dem Lagerbild und Namen im Fächer rechteckig statt oval
- Tests (80): Test-Knöpfe, Material wandert von selbst ins Lager; Doku; 4.9.0

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117M4aYJ5RoPwj7oU8m6XcB
</commit_message>
<xml_diff>
--- a/data/welt.xlsx
+++ b/data/welt.xlsx
@@ -3445,7 +3445,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
@@ -3564,7 +3564,7 @@
         <v>2</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>20</v>
@@ -3603,7 +3603,7 @@
         <v>2</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>20</v>
@@ -3626,7 +3626,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Aufbewahrung</t>
+          <t>Krempelplatz</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
@@ -3642,7 +3642,7 @@
         <v>3</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>6</v>
@@ -3681,7 +3681,7 @@
         <v>3</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="n">
@@ -4475,7 +4475,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Hygge, die das Lager braucht, bevor es auf die nächste Stufe ausgebaut werden kann. Hygge ist die Summe der Einrichtungen. Der Ausbau selbst folgt später.</t>
+          <t>Hygge, ab der das Lager auf die nächste Stufe aufgewertet werden kann (kein Muss). Hygge ist die Summe der Einrichtungen, später auch der Deko. Jede Stufe verlangt mehr. Das Aufwerten selbst folgt später.</t>
         </is>
       </c>
     </row>
@@ -4490,12 +4490,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>id, name</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>steinlager, pilzlager, aufbewahrung, schlafplatz. Jede Einrichtung gibt es in Stufen; jede Zeile ist eine Stufe.</t>
+          <t>id: steinlager, pilzlager, aufbewahrung, schlafplatz. Jede Einrichtung gibt es in Stufen; jede Zeile ist eine Stufe und kann ihren eigenen Namen haben (die Aufbewahrung heißt auf Stufe 1 Krempelplatz).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deko-Liste: Hängematte und Schlafmatte entfernt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117M4aYJ5RoPwj7oU8m6XcB
</commit_message>
<xml_diff>
--- a/data/welt.xlsx
+++ b/data/welt.xlsx
@@ -3704,7 +3704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3762,55 +3762,55 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>schlafmatte</t>
+          <t>wasserkrug</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Schlafmatte</t>
+          <t>Wasserkrug</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>erholung:+8</t>
+          <t>erholung:+4</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>haendler</t>
+          <t>haendler, beute</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>2</v>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Dick genug, um den Boden zu vergessen.</t>
+          <t>Immer kühl, immer gefüllt.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>icon_einrichtung_schlafmatte.png</t>
+          <t>icon_einrichtung_wasserkrug.png</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>wasserkrug</t>
+          <t>kraeuterbund</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Wasserkrug</t>
+          <t>Kräuterbund</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>erholung:+4</t>
+          <t>erholung:+5</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -3819,117 +3819,117 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>2</v>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Immer kühl, immer gefüllt.</t>
+          <t>Riecht nach einem Sommer, den es hier nie gab.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>icon_einrichtung_wasserkrug.png</t>
+          <t>icon_einrichtung_kraeuterbund.png</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>kraeuterbund</t>
+          <t>laterne</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Kräuterbund</t>
+          <t>Laterne</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>erholung:+5</t>
+          <t>glueck:+3</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>haendler, beute</t>
+          <t>haendler</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>2</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Riecht nach einem Sommer, den es hier nie gab.</t>
+          <t>Wirft ein ruhiges Licht.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>icon_einrichtung_kraeuterbund.png</t>
+          <t>icon_einrichtung_laterne.png</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>laterne</t>
+          <t>windspiel</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Laterne</t>
+          <t>Windspiel</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>glueck:+3</t>
+          <t>glueck:+5</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>haendler</t>
+          <t>beute, quest</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>2</v>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Wirft ein ruhiges Licht.</t>
+          <t>Klingt, bevor sich das Wetter ändert.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>icon_einrichtung_laterne.png</t>
+          <t>icon_einrichtung_windspiel.png</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>windspiel</t>
+          <t>wolldecke</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Windspiel</t>
+          <t>Wolldecke</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>glueck:+5</t>
+          <t>erholung:+5</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>beute, quest</t>
+          <t>beute</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
@@ -3940,67 +3940,67 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Klingt, bevor sich das Wetter ändert.</t>
+          <t>Schwer und warm.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>icon_einrichtung_windspiel.png</t>
+          <t>icon_einrichtung_wolldecke.png</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>wolldecke</t>
+          <t>teppich</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Wolldecke</t>
+          <t>Teppich</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>erholung:+5</t>
+          <t>erholung:+6, glueck:+2</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>beute</t>
+          <t>haendler</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Schwer und warm.</t>
+          <t>Muster, in denen man sich verlieren kann.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>icon_einrichtung_wolldecke.png</t>
+          <t>icon_einrichtung_teppich.png</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>haengematte</t>
+          <t>regal</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Hängematte</t>
+          <t>Steinregal</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>erholung:+10</t>
+          <t>glueck:+4</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -4009,36 +4009,36 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>3</v>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Schaukelt noch, wenn man längst schläft.</t>
+          <t>Für alles, was man unterwegs findet.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>icon_einrichtung_haengematte.png</t>
+          <t>icon_einrichtung_regal.png</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>teppich</t>
+          <t>kamin</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Teppich</t>
+          <t>Kamin</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>erholung:+6, glueck:+2</t>
+          <t>erholung:+15</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -4047,131 +4047,55 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Muster, in denen man sich verlieren kann.</t>
+          <t>Das Feuer zieht, der Rauch geht hinaus.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>icon_einrichtung_teppich.png</t>
+          <t>icon_einrichtung_kamin.png</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>regal</t>
+          <t>splitterschale</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Steinregal</t>
+          <t>Splitterschale</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>glueck:+4</t>
+          <t>glueck:+8</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>haendler</t>
+          <t>quest</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Für alles, was man unterwegs findet.</t>
+          <t>Eine Schale voller Bannsplitter, die nie ganz erlöschen.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>icon_einrichtung_regal.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>kamin</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Kamin</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>erholung:+15</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>haendler</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="n">
-        <v>150</v>
-      </c>
-      <c r="F11" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>Das Feuer zieht, der Rauch geht hinaus.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>icon_einrichtung_kamin.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>splitterschale</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Splitterschale</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>glueck:+8</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>quest</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>Eine Schale voller Bannsplitter, die nie ganz erlöschen.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>icon_einrichtung_splitterschale.png</t>
         </is>

</xml_diff>

<commit_message>
Lager: Steinpferch statt Steinkiste, Zeichnungen der Lager Stufe 2
- Steinlager Stufe 2 heißt jetzt Steinpferch („Ein Pferch aus
  Pilzholzstielen, damit der Haufen nicht auseinanderrollt.“), passend
  zur Zeichnung der Nutzerin. welt.xlsx neu aus dem Generator (vorher
  geprüft: unverändert gegenüber dem Generator).
- Die Zeichnungen von Steinpferch und Pilzholzgestell liegen im Lagerbild.
- Version 4.15.5.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117M4aYJ5RoPwj7oU8m6XcB
</commit_message>
<xml_diff>
--- a/data/welt.xlsx
+++ b/data/welt.xlsx
@@ -3714,7 +3714,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Steinkiste</t>
+          <t>Steinpferch</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
@@ -3738,7 +3738,7 @@
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Eine Kiste aus Pilzholz, mit Steinen beschwert, damit der Deckel hält.</t>
+          <t>Ein Pferch aus Pilzholzstielen, damit der Haufen nicht auseinanderrollt.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Start ohne Handschuhe, Handwickel aus einer Quest, Rundgang zum Tageswerk
- Der Envoy beginnt ohne Handschuhe. Die ersten Handwickel bringt die Quest
  „Stoff zwischen den Trümmern“ auf dem Trümmerfeld (ohne Voraussetzung,
  2 Energie, kein Weg); das Lagerfeuer bleibt am ersten Tag sicher machbar
- Die Handwickel tragen jetzt die Zeichnungen der Nutzerin (Nr. 7 und 8 der
  Kleiderkammer, auf 1024 × 1536 vergrößert), mit Icons für beide Figuren
- Rundgang der Envoy-Seite mit fünftem Schritt auf den Tageswerk-Knopf
- Neuer Rundgang beim ersten Öffnen des Tageswerks (drei Schritte)
- Tabellen über den Generator, Tests, CLAUDE.md, Spezifikation; Version 5.5.0

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117M4aYJ5RoPwj7oU8m6XcB
</commit_message>
<xml_diff>
--- a/data/welt.xlsx
+++ b/data/welt.xlsx
@@ -1818,7 +1818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P24"/>
+  <dimension ref="A1:P25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2357,17 +2357,17 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>q-uferkies</t>
+          <t>q-handwickel</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Splitter im Uferkies</t>
+          <t>Stoff zwischen den Trümmern</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>stillesufer</t>
+          <t>truemmerfeld</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -2377,29 +2377,25 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Wo früher Geister gebannt wurden, glimmen noch Splitter zwischen den Kieseln.</t>
+          <t>Unter einer umgestürzten Säule klemmt ein langer Streifen Leinen. Um die Hände gewickelt, schützt er die Knöchel.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr"/>
       <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>gelassenheit</t>
-        </is>
-      </c>
+      <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>splitter:1</t>
+          <t>item:handschuhe_handwickel_1</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nein</t>
         </is>
       </c>
       <c r="N9" s="2" t="n">
@@ -2415,12 +2411,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>q-saeule</t>
+          <t>q-uferkies</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Die umgestürzte Säule</t>
+          <t>Splitter im Uferkies</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2435,32 +2431,24 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Eine Säule liegt quer über dem Pfad. Wer sie zerlegt, hat Stein für Tage.</t>
+          <t>Wo früher Geister gebannt wurden, glimmen noch Splitter zwischen den Kieseln.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>kraft&gt;=3</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>kraft</t>
-        </is>
-      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>kraft</t>
+          <t>gelassenheit</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>stein:4-6, splitter:4</t>
+          <t>splitter:1</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -2469,7 +2457,7 @@
         </is>
       </c>
       <c r="N10" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -2481,57 +2469,61 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>q-haendler</t>
+          <t>q-saeule</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Der Händler im Nebel</t>
+          <t>Die umgestürzte Säule</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>nebelfurt</t>
+          <t>stillesufer</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>kampf</t>
+          <t>erkunden</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>In der Furt ruft jemand um Hilfe. Ein Wagen steckt fest, und davor steht etwas Großes.</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>nebelwaechter</t>
-        </is>
-      </c>
+          <t>Eine Säule liegt quer über dem Pfad. Wer sie zerlegt, hat Stein für Tage.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>kraft&gt;=3, ausdauer&gt;=3</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr"/>
+          <t>kraft&gt;=3</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>kraft</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>kraft</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>freischaltung:haendler, splitter:25</t>
+          <t>stein:4-6, splitter:4</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>nein</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -2543,12 +2535,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>q-furtwache</t>
+          <t>q-haendler</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Wache an der Furt</t>
+          <t>Der Händler im Nebel</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -2558,46 +2550,42 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>erkunden</t>
+          <t>kampf</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Lange am Wasser sitzen, bis der Nebel zeigt, was er mit sich trägt.</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr"/>
+          <t>In der Furt ruft jemand um Hilfe. Ein Wagen steckt fest, und davor steht etwas Großes.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>nebelwaechter</t>
+        </is>
+      </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>gelassenheit&gt;=5</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>gelassenheit</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>gelassenheit</t>
-        </is>
-      </c>
+          <t>kraft&gt;=3, ausdauer&gt;=3</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="n">
-        <v>40</v>
+        <v>6</v>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>splitter:9-12</t>
+          <t>freischaltung:haendler, splitter:25</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nein</t>
         </is>
       </c>
       <c r="N12" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -2609,48 +2597,52 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>q-echohoehle</t>
+          <t>q-furtwache</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Die Echohöhle</t>
+          <t>Wache an der Furt</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>echohoehle</t>
+          <t>nebelfurt</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>hoehle</t>
+          <t>erkunden</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Tief drinnen hausen fünf Geister. Wie weit der Envoy kommt, hängt an den Werten.</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>zauderling, nebelwicht, gruebelkraehe, hastwind, dornenfluesterer</t>
-        </is>
-      </c>
+          <t>Lange am Wasser sitzen, bis der Nebel zeigt, was er mit sich trägt.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr"/>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>kraft&gt;=2</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
+          <t>gelassenheit&gt;=5</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>gelassenheit</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>gelassenheit</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="n">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>splitter:30, item:beine_kampfhose_2</t>
+          <t>splitter:9-12</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -2659,7 +2651,7 @@
         </is>
       </c>
       <c r="N13" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -2671,61 +2663,57 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>q-spalt</t>
+          <t>q-echohoehle</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Durch den Spalt</t>
+          <t>Die Echohöhle</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>spalt</t>
+          <t>echohoehle</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>erkunden</t>
+          <t>hoehle</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Dahinter soll ein Versteck liegen. Hindurch passt nur, wer sich drehen und strecken kann.</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr"/>
+          <t>Tief drinnen hausen fünf Geister. Wie weit der Envoy kommt, hängt an den Werten.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>zauderling, nebelwicht, gruebelkraehe, hastwind, dornenfluesterer</t>
+        </is>
+      </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>beweglichkeit&gt;=4</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>beweglichkeit</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>beweglichkeit</t>
-        </is>
-      </c>
+          <t>kraft&gt;=2</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="n">
         <v>12</v>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>splitter:15, item:kopf_stirnband_1</t>
+          <t>splitter:30, item:beine_kampfhose_2</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>nein</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -2737,17 +2725,17 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>q-quelle</t>
+          <t>q-spalt</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Die stille Quelle</t>
+          <t>Durch den Spalt</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>stillequelle</t>
+          <t>spalt</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -2757,41 +2745,41 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Wer am Rand sitzen bleibt, bis das Wasser ganz ruhig ist, steht erholt wieder auf.</t>
+          <t>Dahinter soll ein Versteck liegen. Hindurch passt nur, wer sich drehen und strecken kann.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr"/>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>gelassenheit&gt;=3</t>
+          <t>beweglichkeit&gt;=4</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>gelassenheit</t>
+          <t>beweglichkeit</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>gelassenheit</t>
+          <t>beweglichkeit</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>splitter:8, rast:1</t>
+          <t>splitter:15, item:kopf_stirnband_1</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nein</t>
         </is>
       </c>
       <c r="N15" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -2803,17 +2791,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>q-dornen</t>
+          <t>q-quelle</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Über den Dornengrat</t>
+          <t>Die stille Quelle</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>dornengrat</t>
+          <t>stillequelle</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -2823,18 +2811,18 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Der Grat flüstert. Hinüber kommt, wer sich weder hetzen noch festhalten lässt.</t>
+          <t>Wer am Rand sitzen bleibt, bis das Wasser ganz ruhig ist, steht erholt wieder auf.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>beweglichkeit&gt;=5, gelassenheit&gt;=4</t>
+          <t>gelassenheit&gt;=3</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>beweglichkeit</t>
+          <t>gelassenheit</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -2844,20 +2832,20 @@
       </c>
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>splitter:20</t>
+          <t>splitter:8, rast:1</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>nein</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -2869,52 +2857,52 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>q-bruecke</t>
+          <t>q-dornen</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Die Brücke über die Schlucht</t>
+          <t>Über den Dornengrat</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>schlucht</t>
+          <t>dornengrat</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>bauen</t>
+          <t>erkunden</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Mit Pilzholz, Stein und einem langen Atem lässt sich die Brücke neu legen.</t>
+          <t>Der Grat flüstert. Hinüber kommt, wer sich weder hetzen noch festhalten lässt.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>ausdauer&gt;=5, kraft&gt;=4</t>
+          <t>beweglichkeit&gt;=5, gelassenheit&gt;=4</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>kraft, ausdauer</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr"/>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>pilzholz:10, stein:12</t>
-        </is>
-      </c>
+          <t>beweglichkeit</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>gelassenheit</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>splitter:30, item:handschuhe_griffhandschuhe_2</t>
+          <t>splitter:20</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
@@ -2935,48 +2923,52 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>q-mondsee</t>
+          <t>q-bruecke</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Spiegel im Mondsee</t>
+          <t>Die Brücke über die Schlucht</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>mondsee</t>
+          <t>schlucht</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>kampf</t>
+          <t>bauen</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Im Wasser steht jemand, der nur wiederholt, was man selbst einmal gesagt hat.</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>echo</t>
-        </is>
-      </c>
+          <t>Mit Pilzholz, Stein und einem langen Atem lässt sich die Brücke neu legen.</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>gelassenheit&gt;=6</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr"/>
+          <t>ausdauer&gt;=5, kraft&gt;=4</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>kraft, ausdauer</t>
+        </is>
+      </c>
       <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>pilzholz:10, stein:12</t>
+        </is>
+      </c>
       <c r="K18" s="2" t="n">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>splitter:35, item:kopf_stillemaske_3</t>
+          <t>splitter:30, item:handschuhe_griffhandschuhe_2</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -2997,12 +2989,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>q-mondnacht</t>
+          <t>q-mondsee</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Eine Nacht am Mondsee</t>
+          <t>Spiegel im Mondsee</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -3012,46 +3004,42 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>erkunden</t>
+          <t>kampf</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Bis der Mond über das Wasser gewandert ist. Was dann im Uferschlamm liegt, hat lange gewartet.</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr"/>
+          <t>Im Wasser steht jemand, der nur wiederholt, was man selbst einmal gesagt hat.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>echo</t>
+        </is>
+      </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>quest:q-mondsee</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>gelassenheit</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>gelassenheit</t>
-        </is>
-      </c>
+          <t>gelassenheit&gt;=6</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="n">
-        <v>60</v>
+        <v>6</v>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>splitter:15-19</t>
+          <t>splitter:35, item:kopf_stillemaske_3</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nein</t>
         </is>
       </c>
       <c r="N19" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -3063,17 +3051,17 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>q-turm</t>
+          <t>q-mondnacht</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Der Turm der Stufen</t>
+          <t>Eine Nacht am Mondsee</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>turm</t>
+          <t>mondsee</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -3083,41 +3071,41 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Oben soll man weit sehen. Wer im echten Leben genug Stufen gegangen ist, kennt den Rhythmus.</t>
+          <t>Bis der Mond über das Wasser gewandert ist. Was dann im Uferschlamm liegt, hat lange gewartet.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>summe_treppe_min&gt;=60</t>
+          <t>quest:q-mondsee</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>ausdauer</t>
+          <t>gelassenheit</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>ausdauer</t>
+          <t>gelassenheit</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>splitter:60, item:schuhe_leichtestiefel_3</t>
+          <t>splitter:15-19</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>nein</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -3129,17 +3117,17 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>q-langestrasse</t>
+          <t>q-turm</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Die lange Straße</t>
+          <t>Der Turm der Stufen</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>langestrasse</t>
+          <t>turm</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -3149,13 +3137,13 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Die Straße endet nur für die, die schon viele Stufen in den Beinen haben.</t>
+          <t>Oben soll man weit sehen. Wer im echten Leben genug Stufen gegangen ist, kennt den Rhythmus.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr"/>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>summe_treppe_min&gt;=150</t>
+          <t>summe_treppe_min&gt;=60</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -3170,11 +3158,11 @@
       </c>
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>splitter:40</t>
+          <t>splitter:60, item:schuhe_leichtestiefel_3</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
@@ -3195,12 +3183,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>q-horizont</t>
+          <t>q-langestrasse</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Bis zum Horizont</t>
+          <t>Die lange Straße</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -3215,13 +3203,13 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Hinter dem Ende der Straße geht es weiter. Wer bis zum Abend läuft, kommt mit vollen Taschen zurück.</t>
+          <t>Die Straße endet nur für die, die schon viele Stufen in den Beinen haben.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>quest:q-langestrasse</t>
+          <t>summe_treppe_min&gt;=150</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -3236,20 +3224,20 @@
       </c>
       <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="n">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>splitter:24-30</t>
+          <t>splitter:40</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nein</t>
         </is>
       </c>
       <c r="N22" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -3261,57 +3249,61 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>q-aschenthron</t>
+          <t>q-horizont</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Der Aschenthron</t>
+          <t>Bis zum Horizont</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>aschenhang</t>
+          <t>langestrasse</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>hoehle</t>
+          <t>erkunden</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Der Weg zum Thron führt an drei Wächtern vorbei. Oben sitzt sie, auf kalter Glut.</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>schwerer-schatten, glutfresser, glutfresser, aschenkoenigin</t>
-        </is>
-      </c>
+          <t>Hinter dem Ende der Straße geht es weiter. Wer bis zum Abend läuft, kommt mit vollen Taschen zurück.</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr"/>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>kraft&gt;=8</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr"/>
-      <c r="I23" s="2" t="inlineStr"/>
+          <t>quest:q-langestrasse</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>ausdauer</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>ausdauer</t>
+        </is>
+      </c>
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="n">
-        <v>25</v>
+        <v>90</v>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>splitter:120, item:handschuhe_nebelwickel_4</t>
+          <t>splitter:24-30</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>nein</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -3323,48 +3315,48 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>q-leere</t>
+          <t>q-aschenthron</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Das weiße Schweigen</t>
+          <t>Der Aschenthron</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>weisstal</t>
+          <t>aschenhang</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>kampf</t>
+          <t>hoehle</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Im Tal wartet etwas, das man nicht besiegen muss.</t>
+          <t>Der Weg zum Thron führt an drei Wächtern vorbei. Oben sitzt sie, auf kalter Glut.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>die-leere</t>
+          <t>schwerer-schatten, glutfresser, glutfresser, aschenkoenigin</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>gelassenheit&gt;=10</t>
+          <t>kraft&gt;=8</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>splitter:200</t>
+          <t>splitter:120, item:handschuhe_nebelwickel_4</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
@@ -3381,6 +3373,68 @@
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>q-leere</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Das weiße Schweigen</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>weisstal</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>kampf</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Im Tal wartet etwas, das man nicht besiegen muss.</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>die-leere</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>gelassenheit&gt;=10</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>splitter:200</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="3">

</xml_diff>

<commit_message>
Start ohne Schuhe, Bastsandalen aus einer Quest im Pilzhain
- Der Envoy beginnt barfuß. Die Bastsandalen bringt die Quest „Bast aus dem
  Pilzhain“ (ohne Voraussetzung, 2 Energie und je 1 Energie Weg)
- Die Bastsandalen tragen die Zeichnung der Nutzerin (Nr. 9 der Kleiderkammer,
  auf 1024 × 1536 vergrößert); sie passt an die Füße beider Figuren
- Tabellen über den Generator, Tests, CLAUDE.md, Spezifikation; Version 5.5.1

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117M4aYJ5RoPwj7oU8m6XcB
</commit_message>
<xml_diff>
--- a/data/welt.xlsx
+++ b/data/welt.xlsx
@@ -1818,7 +1818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1924,12 +1924,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>q-pilzholz-klein</t>
+          <t>q-bastsandalen</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Pilzholz auflesen</t>
+          <t>Bast aus dem Pilzhain</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1939,34 +1939,30 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>sammeln</t>
+          <t>erkunden</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Was der Wind von den Hüten gebrochen hat, liegt leicht im Moos.</t>
+          <t>Die alten Pilzstiele lassen lange, zähe Fasern los. Geflochten und um die Füße gebunden, tragen sie über Stein und Splitter.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>kraft</t>
-        </is>
-      </c>
+      <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>pilzholz:7-9</t>
+          <t>item:schuhe_bastsandalen_1</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nein</t>
         </is>
       </c>
       <c r="N2" s="2" t="n">
@@ -1982,12 +1978,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>q-pilzholz</t>
+          <t>q-pilzholz-klein</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Pilzholz schlagen</t>
+          <t>Pilzholz auflesen</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2002,16 +1998,12 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Einen Stiel fällen und in leichte, handliche Stücke teilen.</t>
+          <t>Was der Wind von den Hüten gebrochen hat, liegt leicht im Moos.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
       <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>kraft, ausdauer</t>
-        </is>
-      </c>
+      <c r="H3" s="2" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr">
         <is>
           <t>kraft</t>
@@ -2019,11 +2011,11 @@
       </c>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>pilzholz:16-20</t>
+          <t>pilzholz:7-9</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -2044,12 +2036,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>q-pilzholz-gross</t>
+          <t>q-pilzholz</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Einen Riesenpilz fällen</t>
+          <t>Pilzholz schlagen</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2064,15 +2056,11 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Ein ganzer Stamm, so hoch wie eine Säule. Das Holz reicht für eine Wand.</t>
+          <t>Einen Stiel fällen und in leichte, handliche Stücke teilen.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>kraft&gt;=4</t>
-        </is>
-      </c>
+      <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
           <t>kraft, ausdauer</t>
@@ -2085,11 +2073,11 @@
       </c>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>pilzholz:38-44</t>
+          <t>pilzholz:16-20</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -2110,17 +2098,17 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>q-stein-klein</t>
+          <t>q-pilzholz-gross</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Lose Steine auflesen</t>
+          <t>Einen Riesenpilz fällen</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>steinbruch</t>
+          <t>pilzhain</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -2130,12 +2118,20 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Am Rand des Bruchs liegt, was von allein herabgefallen ist.</t>
+          <t>Ein ganzer Stamm, so hoch wie eine Säule. Das Holz reicht für eine Wand.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>kraft&gt;=4</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>kraft, ausdauer</t>
+        </is>
+      </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
           <t>kraft</t>
@@ -2143,11 +2139,11 @@
       </c>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>stein:7-9</t>
+          <t>pilzholz:38-44</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -2168,12 +2164,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>q-stein</t>
+          <t>q-stein-klein</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Steine brechen</t>
+          <t>Lose Steine auflesen</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2188,16 +2184,12 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Lose Blöcke lösen und handlich schlagen.</t>
+          <t>Am Rand des Bruchs liegt, was von allein herabgefallen ist.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>kraft</t>
-        </is>
-      </c>
+      <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>kraft</t>
@@ -2205,11 +2197,11 @@
       </c>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>stein:16-20</t>
+          <t>stein:7-9</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -2230,12 +2222,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>q-stein-gross</t>
+          <t>q-stein</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Einen Block lösen</t>
+          <t>Steine brechen</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2250,15 +2242,11 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Ein Block aus der Wand, sauber gespalten. Schwer, aber er trägt ein Haus.</t>
+          <t>Lose Blöcke lösen und handlich schlagen.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>kraft&gt;=5</t>
-        </is>
-      </c>
+      <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr">
         <is>
           <t>kraft</t>
@@ -2271,11 +2259,11 @@
       </c>
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>stein:38-44</t>
+          <t>stein:16-20</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -2296,25 +2284,91 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>q-stein-gross</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Einen Block lösen</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>steinbruch</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>sammeln</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Ein Block aus der Wand, sauber gespalten. Schwer, aber er trägt ein Haus.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>kraft&gt;=5</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>kraft</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>kraft</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>stein:38-44</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>q-lagerfeuer</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Ein Lagerfeuer errichten</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>lager</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>bauen</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Dein Envoy braucht Steine und Pilzholz für das Lagerfeuer. Das kannst du immer in der Gegend sammeln.
 Aber Achtung: Alle Aktivitäten kosten den Envoy Energie. Achte also darauf, dass dein Envoy noch Energie übrig hat, um das Lagerfeuer zu errichten.
@@ -2322,75 +2376,21 @@
 Sammle mit deinem Envoy 8 Steine und 2 Pilzholz, damit er ein Lagerfeuer errichten kann.</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>stein:8, pilzholz:2</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>freischaltung:lagerfeuer</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>nein</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="P8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>q-handwickel</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Stoff zwischen den Trümmern</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>truemmerfeld</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>erkunden</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>Unter einer umgestürzten Säule klemmt ein langer Streifen Leinen. Um die Hände gewickelt, schützt er die Knöchel.</t>
-        </is>
-      </c>
       <c r="F9" s="2" t="inlineStr"/>
       <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>stein:8, pilzholz:2</t>
+        </is>
+      </c>
       <c r="K9" s="2" t="n">
         <v>2</v>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>item:handschuhe_handwickel_1</t>
+          <t>freischaltung:lagerfeuer</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
@@ -2411,17 +2411,17 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>q-uferkies</t>
+          <t>q-handwickel</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Splitter im Uferkies</t>
+          <t>Stoff zwischen den Trümmern</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>stillesufer</t>
+          <t>truemmerfeld</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -2431,29 +2431,25 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Wo früher Geister gebannt wurden, glimmen noch Splitter zwischen den Kieseln.</t>
+          <t>Unter einer umgestürzten Säule klemmt ein langer Streifen Leinen. Um die Hände gewickelt, schützt er die Knöchel.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr"/>
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>gelassenheit</t>
-        </is>
-      </c>
+      <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>splitter:1</t>
+          <t>item:handschuhe_handwickel_1</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nein</t>
         </is>
       </c>
       <c r="N10" s="2" t="n">
@@ -2469,12 +2465,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>q-saeule</t>
+          <t>q-uferkies</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Die umgestürzte Säule</t>
+          <t>Splitter im Uferkies</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -2489,32 +2485,24 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Eine Säule liegt quer über dem Pfad. Wer sie zerlegt, hat Stein für Tage.</t>
+          <t>Wo früher Geister gebannt wurden, glimmen noch Splitter zwischen den Kieseln.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>kraft&gt;=3</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>kraft</t>
-        </is>
-      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>kraft</t>
+          <t>gelassenheit</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>stein:4-6, splitter:4</t>
+          <t>splitter:1</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
@@ -2523,7 +2511,7 @@
         </is>
       </c>
       <c r="N11" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -2535,57 +2523,61 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>q-haendler</t>
+          <t>q-saeule</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Der Händler im Nebel</t>
+          <t>Die umgestürzte Säule</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>nebelfurt</t>
+          <t>stillesufer</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>kampf</t>
+          <t>erkunden</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>In der Furt ruft jemand um Hilfe. Ein Wagen steckt fest, und davor steht etwas Großes.</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>nebelwaechter</t>
-        </is>
-      </c>
+          <t>Eine Säule liegt quer über dem Pfad. Wer sie zerlegt, hat Stein für Tage.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>kraft&gt;=3, ausdauer&gt;=3</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
+          <t>kraft&gt;=3</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>kraft</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>kraft</t>
+        </is>
+      </c>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>freischaltung:haendler, splitter:25</t>
+          <t>stein:4-6, splitter:4</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>nein</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="N12" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -2597,12 +2589,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>q-furtwache</t>
+          <t>q-haendler</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Wache an der Furt</t>
+          <t>Der Händler im Nebel</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -2612,46 +2604,42 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>erkunden</t>
+          <t>kampf</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Lange am Wasser sitzen, bis der Nebel zeigt, was er mit sich trägt.</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr"/>
+          <t>In der Furt ruft jemand um Hilfe. Ein Wagen steckt fest, und davor steht etwas Großes.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>nebelwaechter</t>
+        </is>
+      </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>gelassenheit&gt;=5</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>gelassenheit</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>gelassenheit</t>
-        </is>
-      </c>
+          <t>kraft&gt;=3, ausdauer&gt;=3</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="n">
-        <v>40</v>
+        <v>6</v>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>splitter:9-12</t>
+          <t>freischaltung:haendler, splitter:25</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nein</t>
         </is>
       </c>
       <c r="N13" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -2663,48 +2651,52 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>q-echohoehle</t>
+          <t>q-furtwache</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Die Echohöhle</t>
+          <t>Wache an der Furt</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>echohoehle</t>
+          <t>nebelfurt</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>hoehle</t>
+          <t>erkunden</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Tief drinnen hausen fünf Geister. Wie weit der Envoy kommt, hängt an den Werten.</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>zauderling, nebelwicht, gruebelkraehe, hastwind, dornenfluesterer</t>
-        </is>
-      </c>
+          <t>Lange am Wasser sitzen, bis der Nebel zeigt, was er mit sich trägt.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>kraft&gt;=2</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
+          <t>gelassenheit&gt;=5</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>gelassenheit</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>gelassenheit</t>
+        </is>
+      </c>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="n">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>splitter:30, item:beine_kampfhose_2</t>
+          <t>splitter:9-12</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -2713,7 +2705,7 @@
         </is>
       </c>
       <c r="N14" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -2725,61 +2717,57 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>q-spalt</t>
+          <t>q-echohoehle</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Durch den Spalt</t>
+          <t>Die Echohöhle</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>spalt</t>
+          <t>echohoehle</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>erkunden</t>
+          <t>hoehle</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Dahinter soll ein Versteck liegen. Hindurch passt nur, wer sich drehen und strecken kann.</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr"/>
+          <t>Tief drinnen hausen fünf Geister. Wie weit der Envoy kommt, hängt an den Werten.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>zauderling, nebelwicht, gruebelkraehe, hastwind, dornenfluesterer</t>
+        </is>
+      </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>beweglichkeit&gt;=4</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>beweglichkeit</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>beweglichkeit</t>
-        </is>
-      </c>
+          <t>kraft&gt;=2</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="n">
         <v>12</v>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>splitter:15, item:kopf_stirnband_1</t>
+          <t>splitter:30, item:beine_kampfhose_2</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>nein</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -2791,17 +2779,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>q-quelle</t>
+          <t>q-spalt</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Die stille Quelle</t>
+          <t>Durch den Spalt</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>stillequelle</t>
+          <t>spalt</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -2811,41 +2799,41 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Wer am Rand sitzen bleibt, bis das Wasser ganz ruhig ist, steht erholt wieder auf.</t>
+          <t>Dahinter soll ein Versteck liegen. Hindurch passt nur, wer sich drehen und strecken kann.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>gelassenheit&gt;=3</t>
+          <t>beweglichkeit&gt;=4</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>gelassenheit</t>
+          <t>beweglichkeit</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>gelassenheit</t>
+          <t>beweglichkeit</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>splitter:8, rast:1</t>
+          <t>splitter:15, item:kopf_stirnband_1</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nein</t>
         </is>
       </c>
       <c r="N16" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -2857,17 +2845,17 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>q-dornen</t>
+          <t>q-quelle</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Über den Dornengrat</t>
+          <t>Die stille Quelle</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>dornengrat</t>
+          <t>stillequelle</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -2877,18 +2865,18 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Der Grat flüstert. Hinüber kommt, wer sich weder hetzen noch festhalten lässt.</t>
+          <t>Wer am Rand sitzen bleibt, bis das Wasser ganz ruhig ist, steht erholt wieder auf.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>beweglichkeit&gt;=5, gelassenheit&gt;=4</t>
+          <t>gelassenheit&gt;=3</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>beweglichkeit</t>
+          <t>gelassenheit</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -2898,20 +2886,20 @@
       </c>
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>splitter:20</t>
+          <t>splitter:8, rast:1</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>nein</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -2923,52 +2911,52 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>q-bruecke</t>
+          <t>q-dornen</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Die Brücke über die Schlucht</t>
+          <t>Über den Dornengrat</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>schlucht</t>
+          <t>dornengrat</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>bauen</t>
+          <t>erkunden</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Mit Pilzholz, Stein und einem langen Atem lässt sich die Brücke neu legen.</t>
+          <t>Der Grat flüstert. Hinüber kommt, wer sich weder hetzen noch festhalten lässt.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>ausdauer&gt;=5, kraft&gt;=4</t>
+          <t>beweglichkeit&gt;=5, gelassenheit&gt;=4</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>kraft, ausdauer</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>pilzholz:10, stein:12</t>
-        </is>
-      </c>
+          <t>beweglichkeit</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>gelassenheit</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>splitter:30, item:handschuhe_griffhandschuhe_2</t>
+          <t>splitter:20</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -2989,48 +2977,52 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>q-mondsee</t>
+          <t>q-bruecke</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Spiegel im Mondsee</t>
+          <t>Die Brücke über die Schlucht</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>mondsee</t>
+          <t>schlucht</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>kampf</t>
+          <t>bauen</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Im Wasser steht jemand, der nur wiederholt, was man selbst einmal gesagt hat.</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>echo</t>
-        </is>
-      </c>
+          <t>Mit Pilzholz, Stein und einem langen Atem lässt sich die Brücke neu legen.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr"/>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>gelassenheit&gt;=6</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr"/>
+          <t>ausdauer&gt;=5, kraft&gt;=4</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>kraft, ausdauer</t>
+        </is>
+      </c>
       <c r="I19" s="2" t="inlineStr"/>
-      <c r="J19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>pilzholz:10, stein:12</t>
+        </is>
+      </c>
       <c r="K19" s="2" t="n">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>splitter:35, item:kopf_stillemaske_3</t>
+          <t>splitter:30, item:handschuhe_griffhandschuhe_2</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
@@ -3051,12 +3043,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>q-mondnacht</t>
+          <t>q-mondsee</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Eine Nacht am Mondsee</t>
+          <t>Spiegel im Mondsee</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -3066,46 +3058,42 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>erkunden</t>
+          <t>kampf</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Bis der Mond über das Wasser gewandert ist. Was dann im Uferschlamm liegt, hat lange gewartet.</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr"/>
+          <t>Im Wasser steht jemand, der nur wiederholt, was man selbst einmal gesagt hat.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>echo</t>
+        </is>
+      </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>quest:q-mondsee</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>gelassenheit</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>gelassenheit</t>
-        </is>
-      </c>
+          <t>gelassenheit&gt;=6</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="n">
-        <v>60</v>
+        <v>6</v>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>splitter:15-19</t>
+          <t>splitter:35, item:kopf_stillemaske_3</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nein</t>
         </is>
       </c>
       <c r="N20" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -3117,17 +3105,17 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>q-turm</t>
+          <t>q-mondnacht</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Der Turm der Stufen</t>
+          <t>Eine Nacht am Mondsee</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>turm</t>
+          <t>mondsee</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -3137,41 +3125,41 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Oben soll man weit sehen. Wer im echten Leben genug Stufen gegangen ist, kennt den Rhythmus.</t>
+          <t>Bis der Mond über das Wasser gewandert ist. Was dann im Uferschlamm liegt, hat lange gewartet.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr"/>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>summe_treppe_min&gt;=60</t>
+          <t>quest:q-mondsee</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>ausdauer</t>
+          <t>gelassenheit</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>ausdauer</t>
+          <t>gelassenheit</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>splitter:60, item:schuhe_leichtestiefel_3</t>
+          <t>splitter:15-19</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>nein</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="N21" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -3183,17 +3171,17 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>q-langestrasse</t>
+          <t>q-turm</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Die lange Straße</t>
+          <t>Der Turm der Stufen</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>langestrasse</t>
+          <t>turm</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -3203,13 +3191,13 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Die Straße endet nur für die, die schon viele Stufen in den Beinen haben.</t>
+          <t>Oben soll man weit sehen. Wer im echten Leben genug Stufen gegangen ist, kennt den Rhythmus.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>summe_treppe_min&gt;=150</t>
+          <t>summe_treppe_min&gt;=60</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -3224,11 +3212,11 @@
       </c>
       <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>splitter:40</t>
+          <t>splitter:60, item:schuhe_leichtestiefel_3</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -3249,12 +3237,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>q-horizont</t>
+          <t>q-langestrasse</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Bis zum Horizont</t>
+          <t>Die lange Straße</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -3269,13 +3257,13 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Hinter dem Ende der Straße geht es weiter. Wer bis zum Abend läuft, kommt mit vollen Taschen zurück.</t>
+          <t>Die Straße endet nur für die, die schon viele Stufen in den Beinen haben.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr"/>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>quest:q-langestrasse</t>
+          <t>summe_treppe_min&gt;=150</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -3290,20 +3278,20 @@
       </c>
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="n">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>splitter:24-30</t>
+          <t>splitter:40</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nein</t>
         </is>
       </c>
       <c r="N23" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -3315,57 +3303,61 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>q-aschenthron</t>
+          <t>q-horizont</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Der Aschenthron</t>
+          <t>Bis zum Horizont</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>aschenhang</t>
+          <t>langestrasse</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>hoehle</t>
+          <t>erkunden</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Der Weg zum Thron führt an drei Wächtern vorbei. Oben sitzt sie, auf kalter Glut.</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>schwerer-schatten, glutfresser, glutfresser, aschenkoenigin</t>
-        </is>
-      </c>
+          <t>Hinter dem Ende der Straße geht es weiter. Wer bis zum Abend läuft, kommt mit vollen Taschen zurück.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>kraft&gt;=8</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr"/>
-      <c r="I24" s="2" t="inlineStr"/>
+          <t>quest:q-langestrasse</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>ausdauer</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>ausdauer</t>
+        </is>
+      </c>
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="n">
-        <v>25</v>
+        <v>90</v>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>splitter:120, item:handschuhe_nebelwickel_4</t>
+          <t>splitter:24-30</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>nein</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -3377,48 +3369,48 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>q-leere</t>
+          <t>q-aschenthron</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Das weiße Schweigen</t>
+          <t>Der Aschenthron</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>weisstal</t>
+          <t>aschenhang</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>kampf</t>
+          <t>hoehle</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Im Tal wartet etwas, das man nicht besiegen muss.</t>
+          <t>Der Weg zum Thron führt an drei Wächtern vorbei. Oben sitzt sie, auf kalter Glut.</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>die-leere</t>
+          <t>schwerer-schatten, glutfresser, glutfresser, aschenkoenigin</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>gelassenheit&gt;=10</t>
+          <t>kraft&gt;=8</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr"/>
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr"/>
       <c r="K25" s="2" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>splitter:200</t>
+          <t>splitter:120, item:handschuhe_nebelwickel_4</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
@@ -3435,6 +3427,68 @@
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>q-leere</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Das weiße Schweigen</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>weisstal</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>kampf</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Im Tal wartet etwas, das man nicht besiegen muss.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>die-leere</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>gelassenheit&gt;=10</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>splitter:200</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="3">

</xml_diff>

<commit_message>
5.13: Arena ohne Energie, Händler früher, Tränke, Kleidung mit Güte und Boni
- Arena: eine Herausforderung kostet keine Energie mehr (ältere Kämpfe ohne Feld
  energie behalten 5)
- Quest „Der Händler im Nebel“ ohne Voraussetzung, am ersten Tag zu schaffen
- Händler: jeden Tag je zwei Pilztee (+10) und Quellsud (+25), beim Kauf getrunken,
  nie über das Ende der Leiste
- Kleidung, die gefunden, erbeutet oder angeboten wird, hat eine Güte (schlicht, gut,
  selten, prächtig) mit 0 bis 3 gewürfelten Boni (Schaden, Treffer, Ausweichen,
  Beruhigen, Erholung, Glück), größer bei stärkerem Envoy; nie ein Stat
- Rahmen in der Farbe der Güte, Boni in allen Fenstern, Preise je Bonus höher
- Neuigkeiten, Handbuch, Spezifikation, CLAUDE.md

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117M4aYJ5RoPwj7oU8m6XcB
</commit_message>
<xml_diff>
--- a/data/welt.xlsx
+++ b/data/welt.xlsx
@@ -1462,16 +1462,16 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -2617,11 +2617,7 @@
           <t>nebelwaechter</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>kraft&gt;=3, ausdauer&gt;=3</t>
-        </is>
-      </c>
+      <c r="G13" s="2" t="inlineStr"/>
       <c r="H13" s="2" t="inlineStr"/>
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
5.19: Quests lohnen sich mehr, das Lager wächst leichter
- Erkunden-Quests (und die Brücke) bringen etwa zwei Bannsplitter je Energie
  statt einen: Uferkies 6–8, Säule 14–18, Stille Quelle 20–24, Wache an der
  Furt 72–88, Nacht am Mondsee 110–130, Bis zum Horizont 170–200; einmalige
  doppelt (welt.xlsx über den Generator, mit dem Einverständnis der Nutzerin)
- Kleidung, die unterwegs gefunden wird, hat die Güte wie bei Geistern
  (35/40/19/6 statt 55/30/12/3)
- Lager aufwerten: 15, 40, 85, 140 Energie am Stück statt 30, 70, 115, 165;
  die erste passt in eine volle Leiste mit Ausdauer 2
- Neuigkeiten (alles seit 5.15), Spezifikation, CLAUDE.md, Tests

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117M4aYJ5RoPwj7oU8m6XcB
</commit_message>
<xml_diff>
--- a/data/welt.xlsx
+++ b/data/welt.xlsx
@@ -2502,7 +2502,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>splitter:3-4</t>
+          <t>splitter:6-8</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
@@ -2568,7 +2568,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>stein:4-6, splitter:7-9</t>
+          <t>stein:4-6, splitter:14-18</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>splitter:36-44</t>
+          <t>splitter:72-88</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -2820,7 +2820,7 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>splitter:15, item:kopf_stirnband_1</t>
+          <t>splitter:30, item:kopf_stirnband_1</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>splitter:10-12, rast:1</t>
+          <t>splitter:20-24, rast:1</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
@@ -2952,7 +2952,7 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>splitter:20</t>
+          <t>splitter:40</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -3018,7 +3018,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>splitter:30, item:handschuhe_griffhandschuhe_2</t>
+          <t>splitter:60, item:handschuhe_griffhandschuhe_2</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>splitter:55-65</t>
+          <t>splitter:110-130</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
@@ -3212,7 +3212,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>splitter:60, item:schuhe_leichtestiefel_3</t>
+          <t>splitter:120, item:schuhe_leichtestiefel_3</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -3278,7 +3278,7 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>splitter:40</t>
+          <t>splitter:80</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>splitter:85-100</t>
+          <t>splitter:170-200</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
@@ -3576,7 +3576,7 @@
         <v>20</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
@@ -3603,7 +3603,7 @@
         <v>50</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
@@ -3630,7 +3630,7 @@
         <v>80</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
@@ -3657,7 +3657,7 @@
         <v>100</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>165</v>
+        <v>140</v>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
5.20.10: Lichterkette und Pilzkappenschale im Lager, Deko abbauen
Die Pilzkappenschale hat jetzt ihr Bild im Lager. Neue Deko Lichterkette
(Zeichnung der Nutzerin, Stufe 2, 4 Hygge); ihr Plan liegt beim Händler,
ab dem 9. Oktober 2026 jeden Tag sicher (TRADER_PLANS_FROM). Gebaute
Deko lässt sich im Lager abbauen: halbes Material zurück, der Plan
bleibt (Ereignis abbau). Neuigkeiten dazu.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117M4aYJ5RoPwj7oU8m6XcB
</commit_message>
<xml_diff>
--- a/data/welt.xlsx
+++ b/data/welt.xlsx
@@ -4364,7 +4364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4490,56 +4490,62 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>steinbank</t>
+          <t>lichterkette</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Steinbank</t>
+          <t>Lichterkette</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>start</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
+          <t>haendler</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>selten</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>40</v>
+      </c>
       <c r="H3" s="2" t="n">
         <v>4</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Eine Bank aus flachen Steinen, gerade breit genug für zwei.</t>
+          <t>Kleine bunte Lichter, quer übers Lager gespannt.</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>icon_einrichtung_steinbank.png</t>
+          <t>icon_einrichtung_lichterkette.png</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>wasserkrug</t>
+          <t>steinbank</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Wasserkrug</t>
+          <t>Steinbank</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -4550,55 +4556,51 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>stillesufer</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>selten</t>
-        </is>
-      </c>
+          <t>start</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Immer kühl, immer gefüllt.</t>
+          <t>Eine Bank aus flachen Steinen, gerade breit genug für zwei.</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>icon_einrichtung_wasserkrug.png</t>
+          <t>icon_einrichtung_steinbank.png</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>kraeuterbund</t>
+          <t>wasserkrug</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Kräuterbund</t>
+          <t>Wasserkrug</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
         <v>3</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>stillequelle</t>
+          <t>stillesufer</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -4608,34 +4610,34 @@
       </c>
       <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>Riecht nach einem Sommer, den es hier nie gab.</t>
+          <t>Immer kühl, immer gefüllt.</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>icon_einrichtung_kraeuterbund.png</t>
+          <t>icon_einrichtung_wasserkrug.png</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>windspiel</t>
+          <t>kraeuterbund</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Windspiel</t>
+          <t>Kräuterbund</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -4646,12 +4648,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>geister</t>
+          <t>stillequelle</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>sehr selten</t>
+          <t>selten</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -4659,173 +4661,173 @@
         <v>8</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Klingt, bevor sich das Wetter ändert.</t>
+          <t>Riecht nach einem Sommer, den es hier nie gab.</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>icon_einrichtung_windspiel.png</t>
+          <t>icon_einrichtung_kraeuterbund.png</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>teppich</t>
+          <t>windspiel</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Teppich</t>
+          <t>Windspiel</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
         <v>3</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>haendler</t>
+          <t>geister</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>selten</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>120</v>
-      </c>
+          <t>sehr selten</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Muster, in denen man sich verlieren kann.</t>
+          <t>Klingt, bevor sich das Wetter ändert.</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>icon_einrichtung_teppich.png</t>
+          <t>icon_einrichtung_windspiel.png</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>kamin</t>
+          <t>teppich</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Kamin</t>
+          <t>Teppich</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>start</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
+          <t>haendler</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>selten</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>120</v>
+      </c>
       <c r="H8" s="2" t="n">
         <v>10</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Das Feuer zieht, der Rauch geht hinaus.</t>
+          <t>Muster, in denen man sich verlieren kann.</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>icon_einrichtung_kamin.png</t>
+          <t>icon_einrichtung_teppich.png</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>laterne</t>
+          <t>kamin</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Laterne</t>
+          <t>Kamin</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
         <v>4</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>langestrasse</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>sehr selten</t>
-        </is>
-      </c>
+          <t>start</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr"/>
       <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>8</v>
+        <v>60</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Wirft ein ruhiges Licht.</t>
+          <t>Das Feuer zieht, der Rauch geht hinaus.</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>icon_einrichtung_laterne.png</t>
+          <t>icon_einrichtung_kamin.png</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>leuchtmooskasten</t>
+          <t>laterne</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Leuchtmooskasten</t>
+          <t>Laterne</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -4836,7 +4838,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>pilzhain</t>
+          <t>langestrasse</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -4846,84 +4848,82 @@
       </c>
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>Ein Kasten voll Moos, das nachts leise leuchtet.</t>
+          <t>Wirft ein ruhiges Licht.</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>icon_einrichtung_leuchtmooskasten.png</t>
+          <t>icon_einrichtung_laterne.png</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>pilzholztisch</t>
+          <t>leuchtmooskasten</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Pilzholztisch</t>
+          <t>Leuchtmooskasten</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
         <v>4</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>haendler</t>
+          <t>pilzhain</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>selten</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>180</v>
-      </c>
+          <t>sehr selten</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
       <c r="H11" s="2" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="I11" s="2" t="n">
         <v>5</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Ein Tisch aus einem einzigen Pilzstiel.</t>
+          <t>Ein Kasten voll Moos, das nachts leise leuchtet.</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>icon_einrichtung_pilzholztisch.png</t>
+          <t>icon_einrichtung_leuchtmooskasten.png</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>regal</t>
+          <t>pilzholztisch</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Steinregal</t>
+          <t>Pilzholztisch</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -4934,44 +4934,46 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>steinbruch</t>
+          <t>haendler</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>sehr selten</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr"/>
+          <t>selten</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>180</v>
+      </c>
       <c r="H12" s="2" t="n">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>15</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>Für alles, was man unterwegs findet.</t>
+          <t>Ein Tisch aus einem einzigen Pilzstiel.</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>icon_einrichtung_regal.png</t>
+          <t>icon_einrichtung_pilzholztisch.png</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>wandbehang</t>
+          <t>regal</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Wandbehang</t>
+          <t>Steinregal</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -4982,7 +4984,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>q-furtwache</t>
+          <t>steinbruch</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -4995,47 +4997,47 @@
         <v>10</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>Ein Tuch mit einem Muster aus Nebel und Wasser.</t>
+          <t>Für alles, was man unterwegs findet.</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>icon_einrichtung_wandbehang.png</t>
+          <t>icon_einrichtung_regal.png</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>nebelspiegel</t>
+          <t>wandbehang</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Nebelspiegel</t>
+          <t>Wandbehang</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
         <v>4</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>mondsee</t>
+          <t>q-furtwache</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>kostbar</t>
+          <t>sehr selten</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
@@ -5043,31 +5045,31 @@
         <v>10</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>Ein Spiegel, in dem der Nebel stillsteht.</t>
+          <t>Ein Tuch mit einem Muster aus Nebel und Wasser.</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>icon_einrichtung_nebelspiegel.png</t>
+          <t>icon_einrichtung_wandbehang.png</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>sternkarte</t>
+          <t>nebelspiegel</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Sternkarte</t>
+          <t>Nebelspiegel</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -5078,92 +5080,92 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>q-mondnacht</t>
+          <t>mondsee</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>sehr selten</t>
+          <t>kostbar</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr"/>
       <c r="H15" s="2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>Die Sterne über dem Mondsee, Punkt für Punkt.</t>
+          <t>Ein Spiegel, in dem der Nebel stillsteht.</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>icon_einrichtung_sternkarte.png</t>
+          <t>icon_einrichtung_nebelspiegel.png</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>klangschale</t>
+          <t>sternkarte</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Klangschale</t>
+          <t>Sternkarte</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
         <v>4</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>echohoehle</t>
+          <t>q-mondnacht</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>selten</t>
+          <t>sehr selten</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
       <c r="H16" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="I16" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I16" s="2" t="n">
-        <v>30</v>
-      </c>
       <c r="J16" s="2" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>Ein Schlag, und der Ton bleibt lange im Raum.</t>
+          <t>Die Sterne über dem Mondsee, Punkt für Punkt.</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>icon_einrichtung_klangschale.png</t>
+          <t>icon_einrichtung_sternkarte.png</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>splitterschale</t>
+          <t>klangschale</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Splitterschale</t>
+          <t>Klangschale</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -5174,30 +5176,78 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>geister</t>
+          <t>echohoehle</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>kostbar</t>
+          <t>selten</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr"/>
       <c r="H17" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I17" s="2" t="n">
         <v>30</v>
       </c>
       <c r="J17" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>Ein Schlag, und der Ton bleibt lange im Raum.</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>icon_einrichtung_klangschale.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>splitterschale</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Splitterschale</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>geister</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>kostbar</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="J18" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="K17" s="3" t="inlineStr">
+      <c r="K18" s="3" t="inlineStr">
         <is>
           <t>Eine Schale voller Bannsplitter, die nie ganz erlöschen.</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>icon_einrichtung_splitterschale.png</t>
         </is>

</xml_diff>

<commit_message>
5.21: Notizen vom 10. Oktober eingearbeitet
- Anhängen: was die Würfel einer Sammelaktion in der Reihe noch brauchen, bleibt frei
- Timer: Zeit zum Seitenwechsel, leises Klopfen, Töne im Voraus gesetzt (auch bei dunklem Bildschirm), Ton am Ende ohne Timer
- Ausdauer: Treppe im Wechsel mit Laufen auf der Stelle, Knie heben, Ausfallschritten (Spalte gruppe, die App wählt)
- Beweglichkeit: Brücke mit drei Stufen statt knienden Ausfallschritts
- Hampel-Runden: kürzere Abschnitte mit Pausen
- Sammel-Quests an Pilzhain und Steinbruch angeglichen, größere mit Voraussetzung
- Aushang: Kleidungsstück oder Bannsplitter; Händler zahlt ein Sechstel
- Boni: Spanne innerhalb der Güte; Erklärung der Boni beim Zeigen
- Abenteuer mit Reitern (Karte, Aushang, Tiefen, Arena), Lager mit Wegweiser „Draußen“

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117M4aYJ5RoPwj7oU8m6XcB
</commit_message>
<xml_diff>
--- a/data/welt.xlsx
+++ b/data/welt.xlsx
@@ -2006,16 +2006,16 @@
       <c r="H3" s="2" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>kraft</t>
+          <t>beweglichkeit</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>pilzholz:7-9</t>
+          <t>pilzholz:6-8</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -2060,24 +2060,28 @@
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>beweglichkeit&gt;=3</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>kraft, ausdauer</t>
+          <t>beweglichkeit, ausdauer</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>kraft</t>
+          <t>beweglichkeit</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>pilzholz:16-20</t>
+          <t>pilzholz:18-22</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -2124,17 +2128,17 @@
       <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>kraft&gt;=4</t>
+          <t>beweglichkeit&gt;=5</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>kraft, ausdauer</t>
+          <t>beweglichkeit, ausdauer</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>kraft</t>
+          <t>beweglichkeit</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
@@ -2143,7 +2147,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>pilzholz:38-44</t>
+          <t>pilzholz:42-48</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -2197,11 +2201,11 @@
       </c>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>stein:7-9</t>
+          <t>stein:6-8</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -2246,7 +2250,11 @@
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>kraft&gt;=3</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
           <t>kraft</t>
@@ -2259,11 +2267,11 @@
       </c>
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>stein:16-20</t>
+          <t>stein:18-22</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -2329,7 +2337,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>stein:38-44</t>
+          <t>stein:42-48</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">

</xml_diff>